<commit_message>
Update FOA workbook content, formatting, and duplicate-title highlighting
</commit_message>
<xml_diff>
--- a/FOA SETS/Accent-Set.xlsx
+++ b/FOA SETS/Accent-Set.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -611,7 +611,7 @@
           <t>Accent</t>
         </is>
       </c>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>Vanity</t>
         </is>
@@ -625,12 +625,12 @@
         <is>
           <t>FREE SHIPPING
 NAUCALPAN Vanity Set w/ Stool offers a pulled-together look that makes the room feel ready to use and enjoy. This accent vanity is made to fit naturally into the room. A Traditional profile gives the space a refined, approachable look. Crafted with Fabric, Solid Wood, Engineered Wood, then finished in White tones to suit a range of interiors.
-Product Dimensions: 47.5" W x 26"D x 46" H, STOOL: 15.5" W x 15.5"D x 16" H
+Product Dimensions: 47.5"W X 26"D X 46"H, STOOL: 15.5"W X 15.5"D X 16"H
 Features
 - Traditional
 - Felt-lined Top Drawers
 - Bracketed Feet
-Materials: Fabric, Solid Wood, Engineered Wood
+Materials: Fabric, Solid Wood, Engineered Wood.
 Color: White
 Weight: 90.86 lbs</t>
         </is>
@@ -727,7 +727,7 @@
           <t>Accent</t>
         </is>
       </c>
-      <c r="F3" s="5" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>Chair</t>
         </is>
@@ -741,16 +741,15 @@
         <is>
           <t>FREE SHIPPING
 VAUGH Accent Chair w/ Ottoman offers a pulled-together look that makes the room feel ready to use and enjoy. This accent chair is made to fit naturally into the room. A Traditional profile gives the space a refined, approachable look. Crafted with Leatherette, Engineered Wood, then finished in Rustic Brown tones to suit a range of interiors.
-Product Dimensions: 33" W x 30"D x 43 3 or 4" H
+Product Dimensions: 33"W X 30"D X 43 3/4"H
 Features
 - Traditional
 - Button Tufting w/ Nailhead Trim
 - Cabriole Legs
-- Matching Ottoman Available
-Included items and dimensions:
+- Matching Ottoman Available Included items and dimensions:
 - Accent Chair: color: Rustic Brown; dimensions: 33" W x 30"D x 43 3 or 4" H; feature: Traditional
 - Ottoman: color: Rustic Brown; dimensions: 20" W x 20"D x 16" H; feature: Traditional
-Materials: Leatherette, Engineered Wood
+Materials: Leatherette, Engineered Wood.
 Color: Rustic Brown
 Weight: 90.2 lbs</t>
         </is>

</xml_diff>

<commit_message>
Update FOA Excel tags, remove Availability column, and clean SEO titles
</commit_message>
<xml_diff>
--- a/FOA SETS/Accent-Set.xlsx
+++ b/FOA SETS/Accent-Set.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -445,183 +445,188 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC3"/>
+  <dimension ref="A1:AD3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Availability</t>
+          <t>Color</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Color</t>
+          <t>Size</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Size</t>
+          <t>SKU</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>SKU</t>
+          <t>Category</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Category</t>
+          <t>Subcategory</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>Subcategory</t>
+          <t>Title</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>Title</t>
+          <t>Description</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>Description</t>
+          <t>seo title(70char)</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>seo title(70char)</t>
+          <t>seo description(160char)</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>seo description(160char)</t>
+          <t>Name</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>Name</t>
+          <t>Short Description</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
         <is>
-          <t>Short Description</t>
+          <t>Short Description - Red Text</t>
         </is>
       </c>
       <c r="M1" t="inlineStr">
         <is>
-          <t>Short Description - Red Text</t>
+          <t>Item Type</t>
         </is>
       </c>
       <c r="N1" t="inlineStr">
         <is>
-          <t>Item Type</t>
+          <t>Parts for Group Items</t>
         </is>
       </c>
       <c r="O1" t="inlineStr">
         <is>
-          <t>Parts for Group Items</t>
+          <t>Images</t>
         </is>
       </c>
       <c r="P1" t="inlineStr">
         <is>
-          <t>Images</t>
+          <t>East(cost)</t>
         </is>
       </c>
       <c r="Q1" t="inlineStr">
         <is>
-          <t>East(cost)</t>
+          <t>EAST COST (Updated)</t>
         </is>
       </c>
       <c r="R1" t="inlineStr">
         <is>
-          <t>EAST COST (Updated)</t>
+          <t>MSRP</t>
         </is>
       </c>
       <c r="S1" t="inlineStr">
         <is>
-          <t>MSRP</t>
+          <t>Weight (LB)</t>
         </is>
       </c>
       <c r="T1" t="inlineStr">
         <is>
-          <t>Weight (LB)</t>
+          <t>Product Dimension (Inch)</t>
         </is>
       </c>
       <c r="U1" t="inlineStr">
         <is>
-          <t>Product Dimension (Inch)</t>
+          <t>Style</t>
         </is>
       </c>
       <c r="V1" t="inlineStr">
         <is>
-          <t>Style</t>
+          <t>Material</t>
         </is>
       </c>
       <c r="W1" t="inlineStr">
         <is>
-          <t>Material</t>
+          <t>Features</t>
         </is>
       </c>
       <c r="X1" t="inlineStr">
         <is>
-          <t>Features</t>
+          <t>Origin</t>
         </is>
       </c>
       <c r="Y1" t="inlineStr">
         <is>
-          <t>Origin</t>
+          <t>Shipping Length (IN)</t>
         </is>
       </c>
       <c r="Z1" t="inlineStr">
         <is>
-          <t>Shipping Length (IN)</t>
+          <t>Shipping Width (IN)</t>
         </is>
       </c>
       <c r="AA1" t="inlineStr">
         <is>
-          <t>Shipping Width (IN)</t>
+          <t>Shipping Height (IN)</t>
         </is>
       </c>
       <c r="AB1" t="inlineStr">
         <is>
-          <t>Shipping Height (IN)</t>
+          <t>Volume (CUFT)</t>
         </is>
       </c>
       <c r="AC1" t="inlineStr">
         <is>
-          <t>Volume (CUFT)</t>
+          <t>Fixed tags</t>
+        </is>
+      </c>
+      <c r="AD1" t="inlineStr">
+        <is>
+          <t>Variable tags</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="B2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>White</t>
         </is>
       </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>FM7456WH-V-SET</t>
+        </is>
+      </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>FM7456WH-V-SET</t>
+          <t>Accent</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Accent</t>
+          <t>Vanity</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Vanity</t>
+          <t>NAUCALPAN Vanity Set w/ Stool</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
-        <is>
-          <t>NAUCALPAN Vanity Set w/ Stool</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
         <is>
           <t>FREE SHIPPING
 NAUCALPAN Vanity Set w/ Stool offers a pulled-together look that makes the room feel ready to use and enjoy. This accent vanity is made to fit naturally into the room. A Traditional profile gives the space a refined, approachable look. Crafted with Fabric, Solid Wood, Engineered Wood, then finished in White tones to suit a range of interiors.
@@ -635,109 +640,119 @@
 Weight: 90.86 lbs</t>
         </is>
       </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>NAUCALPAN Vanity Set w/ Stool in White | GOODDEGG</t>
+        </is>
+      </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>NAUCALPAN Vanity Set w/ Stool in White | GOODDEGG</t>
+          <t>The NAUCALPAN Vanity w/ Stool brings everyday comfort and function to your space. Shop at GOODDEGG for a great selection and guaranteed lowest prices.</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>The NAUCALPAN Vanity w/ Stool brings everyday comfort and function to your space. Shop at GOODDEGG for a great selection and guaranteed lowest prices.</t>
+          <t>NAUCALPAN</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>NAUCALPAN</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
           <t>Vanity Set w/ Stool</t>
         </is>
       </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Set</t>
+        </is>
+      </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>Set</t>
+          <t>FM7456WH-V-1, FM7456WH-V-2</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>FM7456WH-V-1, FM7456WH-V-2</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
           <t>FM7456WH-V-1.jpg,FM7456WH-V-2.jpg,FM7456WH-V-WB-1.jpg,FM7456WH-V-WB-2.jpg,FM7456WH-V-WB-3.jpg,FM7456WH-V-WB-4.jpg</t>
         </is>
       </c>
-      <c r="Q2" t="n">
+      <c r="P2" t="n">
         <v>209</v>
       </c>
-      <c r="R2" s="1" t="n">
+      <c r="Q2" s="1" t="n">
         <v>229</v>
       </c>
+      <c r="R2" t="n">
+        <v>507</v>
+      </c>
       <c r="S2" t="n">
-        <v>507</v>
-      </c>
-      <c r="T2" t="n">
         <v>90.86</v>
       </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>47.5"W X 26"D X 46"H, STOOL: 15.5"W X 15.5"D X 16"H</t>
+        </is>
+      </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>47.5"W X 26"D X 46"H, STOOL: 15.5"W X 15.5"D X 16"H</t>
+          <t>Traditional</t>
         </is>
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>Traditional</t>
+          <t>Fabric, Solid Wood, Engineered Wood</t>
         </is>
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>Fabric, Solid Wood, Engineered Wood</t>
+          <t>Traditional,White,Fabric, Solid Wood, Engineered Wood,Felt-lined Top Drawers,Bracketed Feet</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>Traditional,White,Fabric, Solid Wood, Engineered Wood,Felt-lined Top Drawers,Bracketed Feet</t>
-        </is>
-      </c>
-      <c r="Y2" t="inlineStr">
-        <is>
           <t>VN</t>
         </is>
       </c>
-      <c r="AC2" t="n">
+      <c r="AB2" t="n">
         <v>12.5</v>
+      </c>
+      <c r="AC2" t="inlineStr">
+        <is>
+          <t>Furniture of America, Quick Ship Furniture, New Arrival, Indoor Furniture</t>
+        </is>
+      </c>
+      <c r="AD2" t="inlineStr">
+        <is>
+          <t>Accent, Vanity, NAUCALPAN</t>
+        </is>
       </c>
     </row>
     <row r="3">
-      <c r="B3" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>Rustic Brown</t>
         </is>
       </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>CM-AC6801BR-SET</t>
+        </is>
+      </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>CM-AC6801BR-SET</t>
+          <t>Accent</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Accent</t>
+          <t>Chair</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Chair</t>
+          <t>VAUGH Accent Chair w/ Ottoman</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
-        <is>
-          <t>VAUGH Accent Chair w/ Ottoman</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
         <is>
           <t>FREE SHIPPING
 VAUGH Accent Chair w/ Ottoman offers a pulled-together look that makes the room feel ready to use and enjoy. This accent chair is made to fit naturally into the room. A Traditional profile gives the space a refined, approachable look. Crafted with Leatherette, Engineered Wood, then finished in Rustic Brown tones to suit a range of interiors.
@@ -754,80 +769,90 @@
 Weight: 90.2 lbs</t>
         </is>
       </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>VAUGH Accent Chair w/ Ottoman in Rustic Brown | GOODDEGG</t>
+        </is>
+      </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>VAUGH Accent Chair w/ Ottoman in Rustic Brown | GOODDEGG</t>
+          <t>The VAUGH Accent Chair w/ Ottoman adds comfortable seating and style to your space. Shop at GOODDEGG for a great selection and guaranteed lowest prices.</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>The VAUGH Accent Chair w/ Ottoman adds comfortable seating and style to your space. Shop at GOODDEGG for a great selection and guaranteed lowest prices.</t>
+          <t>VAUGH</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>VAUGH</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
           <t>Accent Chair w/ Ottoman</t>
         </is>
       </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Set</t>
+        </is>
+      </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Set</t>
+          <t>CM-AC6801BR, CM-AC6801BR-OT</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>CM-AC6801BR, CM-AC6801BR-OT</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
           <t>CM-AC6801BR.jpg,CM-AC6801BR-ARM.jpg,CM-AC6801BR-TEXTURE.jpg</t>
         </is>
       </c>
-      <c r="Q3" t="n">
+      <c r="P3" t="n">
         <v>359</v>
       </c>
-      <c r="R3" s="2" t="n">
+      <c r="Q3" s="2" t="n">
         <v>359</v>
       </c>
+      <c r="R3" t="n">
+        <v>927</v>
+      </c>
       <c r="S3" t="n">
-        <v>927</v>
-      </c>
-      <c r="T3" t="n">
         <v>90.2</v>
       </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>33"W X 30"D X 43 3/4"H</t>
+        </is>
+      </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>33"W X 30"D X 43 3/4"H</t>
+          <t>Traditional</t>
         </is>
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>Traditional</t>
+          <t>Leatherette, Engineered Wood</t>
         </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>Leatherette, Engineered Wood</t>
+          <t>Traditional,Rustic Brown,Leatherette, Engineered Wood,Button Tufting w/ Nailhead Trim,Cabriole Legs,Matching Ottoman Available</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>Traditional,Rustic Brown,Leatherette, Engineered Wood,Button Tufting w/ Nailhead Trim,Cabriole Legs,Matching Ottoman Available</t>
-        </is>
-      </c>
-      <c r="Y3" t="inlineStr">
-        <is>
           <t>CN</t>
         </is>
       </c>
-      <c r="AC3" t="n">
+      <c r="AB3" t="n">
         <v>14.7</v>
+      </c>
+      <c r="AC3" t="inlineStr">
+        <is>
+          <t>Furniture of America, Quick Ship Furniture, New Arrival, Indoor Furniture</t>
+        </is>
+      </c>
+      <c r="AD3" t="inlineStr">
+        <is>
+          <t>Accent, Chair, VAUGH</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>